<commit_message>
Add production deploy verification results
Verified live on Railway after deploy: migrations applied cleanly,
all 5 demo accounts log in, new API routes respond correctly, RI-19/RI-25
fixes confirmed blocking the right actions, document traceability feature
works end-to-end, 50MB upload succeeds, response times normal. All test
data (throwaway projects/documents) created and cleaned up by the
verification scripts themselves — no real user data touched.
</commit_message>
<xml_diff>
--- a/docs/pengujian/Hasil-Pengujian-LPS-EDMS.xlsx
+++ b/docs/pengujian/Hasil-Pengujian-LPS-EDMS.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Unggah Berkas Besar" sheetId="6" r:id="rId6"/>
     <sheet name="Integritas Basis Data" sheetId="7" r:id="rId7"/>
     <sheet name="Ringkasan Naratif" sheetId="8" r:id="rId8"/>
+    <sheet name="Verifikasi Deploy Production" sheetId="9" r:id="rId9"/>
   </sheets>
 </workbook>
 </file>
@@ -4575,4 +4576,235 @@
     <ignoredError numberStoredAsText="1" sqref="A1:A14"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F11"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>kode</v>
+      </c>
+      <c r="B1" t="str">
+        <v>yang_diverifikasi</v>
+      </c>
+      <c r="C1" t="str">
+        <v>cara</v>
+      </c>
+      <c r="D1" t="str">
+        <v>hasil</v>
+      </c>
+      <c r="E1" t="str">
+        <v>kesimpulan</v>
+      </c>
+      <c r="F1" t="str">
+        <v>catatan</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>DPL-01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Build &amp; migrasi database berhasil di production</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Push ke GitHub -&gt; Railway auto-build -&gt; cek log startup</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Build sukses (TypeScript check lolos, semua rute ter-generate). Kedua migrasi baru (add_document_references, document_title_trgm_index) diterapkan otomatis lewat 'prisma migrate deploy' saat start, tanpa error. Server siap dalam 149ms.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Lolos</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>DPL-02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Situs bisa diakses setelah deploy</v>
+      </c>
+      <c r="C3" t="str">
+        <v>GET /login</v>
+      </c>
+      <c r="D3" t="str">
+        <v>HTTP 200</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Lolos</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>DPL-03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Login 5 akun demo dengan password baru (hasil rotasi sebelumnya)</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Login masing-masing role, cek sesi berhasil</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Superadmin, Team Leader, Engineer, Inspector, Client - semua berhasil login (sesi tersimpan)</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Lolos</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>DPL-04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Rute API baru (references, traceability) benar-benar ter-deploy</v>
+      </c>
+      <c r="C5" t="str">
+        <v>GET tanpa login ke kedua rute - harus 401 (rute ada), bukan 404 (rute hilang)</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Keduanya membalas 401 seperti seharusnya. Catatan: log build Railway sempat tidak menampilkan kedua rute ini di ringkasan tabel rute - ternyata cuma keterbatasan tampilan log, rute-nya berfungsi normal.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Lolos</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Sempat menimbulkan kekhawatiran di log build, makanya diverifikasi langsung ke endpoint hidup alih-alih percaya ringkasan log saja.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>DPL-05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>RI-25 (Superadmin diblokir upload dokumen) berfungsi di production</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Superadmin coba upload ke proyek uji sungguhan</v>
+      </c>
+      <c r="D6" t="str">
+        <v>HTTP 403, tidak ada dokumen tercipta</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Lolos</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>DPL-06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>RI-19 (Inspector diblokir approve lewat /status) berfungsi di production</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Inspector coba ubah status dokumen sungguhan jadi APPROVED</v>
+      </c>
+      <c r="D7" t="str">
+        <v>HTTP 403, status dokumen tidak berubah</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Lolos</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>DPL-07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Fitur baru: tautan dokumen (BASED_ON) berfungsi end-to-end di production</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Team Leader buat 2 dokumen uji, tautkan satu ke lainnya, cek metrik traceability proyek</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Tautan berhasil dibuat (HTTP 201), endpoint metrik traceability membalas angka yang masuk akal (totalReferences:1)</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Lolos</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>DPL-08</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Batas unggah 200MB (sebelumnya gagal di atas ~10MB) berfungsi di production</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Unggah berkas 50MB sungguhan ke proyek uji</v>
+      </c>
+      <c r="D9" t="str">
+        <v>HTTP 201 berhasil dalam 6,46 detik</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Lolos</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>DPL-09</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Waktu respons endpoint utama masih wajar setelah deploy</v>
+      </c>
+      <c r="C10" t="str">
+        <v>GET dashboard, pencarian dokumen, daftar proyek (baca saja, data sungguhan)</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Dashboard 250ms, pencarian 115ms, daftar proyek 77ms - semua di bawah 300ms</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Lolos</v>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>DPL-10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Data uji dibersihkan total, tidak ada sisa di data production sungguhan</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Cek daftar proyek untuk nama berawalan ZZZ- (penanda proyek uji)</v>
+      </c>
+      <c r="D11" t="str">
+        <v>0 proyek uji tersisa</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Lolos</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Setiap pengujian di production memakai proyek/dokumen yang dibuat sendiri lalu dihapus lagi di akhir - tidak pernah menyentuh data pengguna sungguhan.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add production 150MB upload and concurrent-load verification results
Both run against live production with real HTTP load: 150MB upload
succeeds (19.89s), and GET-only load tests (dashboard + search) at
5/10/20 concurrent connections show zero errors/timeouts at all levels
-- better than the earlier local test-DB results, likely due to
production's Postgres connection pool config. Site health checked
before and after each pass; no new errors in production logs.
</commit_message>
<xml_diff>
--- a/docs/pengujian/Hasil-Pengujian-LPS-EDMS.xlsx
+++ b/docs/pengujian/Hasil-Pengujian-LPS-EDMS.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Integritas Basis Data" sheetId="7" r:id="rId7"/>
     <sheet name="Ringkasan Naratif" sheetId="8" r:id="rId8"/>
     <sheet name="Verifikasi Deploy Production" sheetId="9" r:id="rId9"/>
+    <sheet name="Beban Konkuren Production" sheetId="10" r:id="rId10"/>
   </sheets>
 </workbook>
 </file>
@@ -1656,6 +1657,283 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L7"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>endpoint</v>
+      </c>
+      <c r="B1" t="str">
+        <v>jumlah_koneksi</v>
+      </c>
+      <c r="C1" t="str">
+        <v>req_per_detik</v>
+      </c>
+      <c r="D1" t="str">
+        <v>throughput_kbs</v>
+      </c>
+      <c r="E1" t="str">
+        <v>latensi_rata2_ms</v>
+      </c>
+      <c r="F1" t="str">
+        <v>latensi_p50_ms</v>
+      </c>
+      <c r="G1" t="str">
+        <v>latensi_p97_5_ms</v>
+      </c>
+      <c r="H1" t="str">
+        <v>latensi_p99_ms</v>
+      </c>
+      <c r="I1" t="str">
+        <v>latensi_max_ms</v>
+      </c>
+      <c r="J1" t="str">
+        <v>total_request</v>
+      </c>
+      <c r="K1" t="str">
+        <v>jumlah_gagal</v>
+      </c>
+      <c r="L1" t="str">
+        <v>jumlah_timeout</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>dashboard</v>
+      </c>
+      <c r="B2" t="str">
+        <v>5</v>
+      </c>
+      <c r="C2" t="str">
+        <v>47.14</v>
+      </c>
+      <c r="D2" t="str">
+        <v>207.7</v>
+      </c>
+      <c r="E2" t="str">
+        <v>105.49</v>
+      </c>
+      <c r="F2" t="str">
+        <v>84</v>
+      </c>
+      <c r="G2" t="str">
+        <v>267</v>
+      </c>
+      <c r="H2" t="str">
+        <v>321</v>
+      </c>
+      <c r="I2" t="str">
+        <v>487</v>
+      </c>
+      <c r="J2" t="str">
+        <v>1414</v>
+      </c>
+      <c r="K2" t="str">
+        <v>0</v>
+      </c>
+      <c r="L2" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>dashboard</v>
+      </c>
+      <c r="B3" t="str">
+        <v>10</v>
+      </c>
+      <c r="C3" t="str">
+        <v>79.14</v>
+      </c>
+      <c r="D3" t="str">
+        <v>348.8</v>
+      </c>
+      <c r="E3" t="str">
+        <v>125.87</v>
+      </c>
+      <c r="F3" t="str">
+        <v>109</v>
+      </c>
+      <c r="G3" t="str">
+        <v>251</v>
+      </c>
+      <c r="H3" t="str">
+        <v>281</v>
+      </c>
+      <c r="I3" t="str">
+        <v>395</v>
+      </c>
+      <c r="J3" t="str">
+        <v>2374</v>
+      </c>
+      <c r="K3" t="str">
+        <v>0</v>
+      </c>
+      <c r="L3" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>dashboard</v>
+      </c>
+      <c r="B4" t="str">
+        <v>20</v>
+      </c>
+      <c r="C4" t="str">
+        <v>113</v>
+      </c>
+      <c r="D4" t="str">
+        <v>498.0</v>
+      </c>
+      <c r="E4" t="str">
+        <v>176.23</v>
+      </c>
+      <c r="F4" t="str">
+        <v>165</v>
+      </c>
+      <c r="G4" t="str">
+        <v>307</v>
+      </c>
+      <c r="H4" t="str">
+        <v>332</v>
+      </c>
+      <c r="I4" t="str">
+        <v>388</v>
+      </c>
+      <c r="J4" t="str">
+        <v>3390</v>
+      </c>
+      <c r="K4" t="str">
+        <v>0</v>
+      </c>
+      <c r="L4" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>search</v>
+      </c>
+      <c r="B5" t="str">
+        <v>5</v>
+      </c>
+      <c r="C5" t="str">
+        <v>59</v>
+      </c>
+      <c r="D5" t="str">
+        <v>1240.0</v>
+      </c>
+      <c r="E5" t="str">
+        <v>84.15</v>
+      </c>
+      <c r="F5" t="str">
+        <v>68</v>
+      </c>
+      <c r="G5" t="str">
+        <v>196</v>
+      </c>
+      <c r="H5" t="str">
+        <v>289</v>
+      </c>
+      <c r="I5" t="str">
+        <v>570</v>
+      </c>
+      <c r="J5" t="str">
+        <v>1770</v>
+      </c>
+      <c r="K5" t="str">
+        <v>0</v>
+      </c>
+      <c r="L5" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>search</v>
+      </c>
+      <c r="B6" t="str">
+        <v>10</v>
+      </c>
+      <c r="C6" t="str">
+        <v>76.2</v>
+      </c>
+      <c r="D6" t="str">
+        <v>1601.6</v>
+      </c>
+      <c r="E6" t="str">
+        <v>130.27</v>
+      </c>
+      <c r="F6" t="str">
+        <v>115</v>
+      </c>
+      <c r="G6" t="str">
+        <v>300</v>
+      </c>
+      <c r="H6" t="str">
+        <v>402</v>
+      </c>
+      <c r="I6" t="str">
+        <v>820</v>
+      </c>
+      <c r="J6" t="str">
+        <v>2286</v>
+      </c>
+      <c r="K6" t="str">
+        <v>0</v>
+      </c>
+      <c r="L6" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>search</v>
+      </c>
+      <c r="B7" t="str">
+        <v>20</v>
+      </c>
+      <c r="C7" t="str">
+        <v>101.4</v>
+      </c>
+      <c r="D7" t="str">
+        <v>2130.9</v>
+      </c>
+      <c r="E7" t="str">
+        <v>195.51</v>
+      </c>
+      <c r="F7" t="str">
+        <v>182</v>
+      </c>
+      <c r="G7" t="str">
+        <v>407</v>
+      </c>
+      <c r="H7" t="str">
+        <v>551</v>
+      </c>
+      <c r="I7" t="str">
+        <v>902</v>
+      </c>
+      <c r="J7" t="str">
+        <v>3042</v>
+      </c>
+      <c r="K7" t="str">
+        <v>0</v>
+      </c>
+      <c r="L7" t="str">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:L7"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I28"/>
@@ -4580,7 +4858,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4764,47 +5042,107 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>DPL-09</v>
+        <v>DPL-08b</v>
       </c>
       <c r="B10" t="str">
-        <v>Waktu respons endpoint utama masih wajar setelah deploy</v>
+        <v>Batas unggah mendekati batas maksimal (150MB dari 200MB yang dijanjikan)</v>
       </c>
       <c r="C10" t="str">
-        <v>GET dashboard, pencarian dokumen, daftar proyek (baca saja, data sungguhan)</v>
+        <v>Unggah berkas 150MB sungguhan ke proyek uji terpisah, lalu dibersihkan</v>
       </c>
       <c r="D10" t="str">
-        <v>Dashboard 250ms, pencarian 115ms, daftar proyek 77ms - semua di bawah 300ms</v>
+        <v>HTTP 201 berhasil dalam 19,89 detik</v>
       </c>
       <c r="E10" t="str">
         <v>Lolos</v>
       </c>
       <c r="F10" t="str">
-        <v/>
+        <v>Proyek &amp; dokumen uji dihapus lagi setelahnya, situs tetap sehat (HTTP 200 di /login) sesudahnya.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
+        <v>DPL-11</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Ketahanan sistem terhadap beban bersamaan (5/10/20 pengguna) di production sungguhan</v>
+      </c>
+      <c r="C11" t="str">
+        <v>autocannon 30 detik per tingkat, GET /api/dashboard (baca saja, tidak mengubah data apa pun)</v>
+      </c>
+      <c r="D11" t="str">
+        <v>0 dari total request gagal/timeout di ketiga tingkat beban. Latensi p99 tertinggi 332ms (di 20 pengguna bersamaan).</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Lolos</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Lebih baik dari hasil di lingkungan uji lokal sebelumnya (yang sempat menunjukkan timeout) — kemungkinan besar karena konfigurasi database production berbeda dari database uji lokal. Situs dicek sehat (HTTP 200) sebelum dan sesudah pengujian ini.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>DPL-12</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Ketahanan fitur pencarian terhadap beban bersamaan (5/10/20 pengguna) di production sungguhan</v>
+      </c>
+      <c r="C12" t="str">
+        <v>autocannon 30 detik per tingkat, GET pencarian dokumen (baca saja)</v>
+      </c>
+      <c r="D12" t="str">
+        <v>0 dari total request gagal/timeout di ketiga tingkat beban. Latensi p99 tertinggi 551ms (di 20 pengguna bersamaan).</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Lolos</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Situs dicek sehat sebelum dan sesudah pengujian ini — tidak ada error baru muncul di log production selama maupun setelah pengujian beban.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>DPL-09</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Waktu respons endpoint utama masih wajar setelah deploy</v>
+      </c>
+      <c r="C13" t="str">
+        <v>GET dashboard, pencarian dokumen, daftar proyek (baca saja, data sungguhan)</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Dashboard 250ms, pencarian 115ms, daftar proyek 77ms - semua di bawah 300ms</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Lolos</v>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
         <v>DPL-10</v>
       </c>
-      <c r="B11" t="str">
+      <c r="B14" t="str">
         <v>Data uji dibersihkan total, tidak ada sisa di data production sungguhan</v>
       </c>
-      <c r="C11" t="str">
+      <c r="C14" t="str">
         <v>Cek daftar proyek untuk nama berawalan ZZZ- (penanda proyek uji)</v>
       </c>
-      <c r="D11" t="str">
+      <c r="D14" t="str">
         <v>0 proyek uji tersisa</v>
       </c>
-      <c r="E11" t="str">
-        <v>Lolos</v>
-      </c>
-      <c r="F11" t="str">
+      <c r="E14" t="str">
+        <v>Lolos</v>
+      </c>
+      <c r="F14" t="str">
         <v>Setiap pengujian di production memakai proyek/dokumen yang dibuat sendiri lalu dihapus lagi di akhir - tidak pernah menyentuh data pengguna sungguhan.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add FR-04 and FR-08 test coverage (previously untested requirements)
FR-04 (per-project role resolution) and FR-08 (auto 6-phase project
creation) had no dedicated test evidence. Both verified via real API
calls against the isolated test DB, both Lolos; consolidated into
hasil-gabungan.csv and the combined xlsx (69/71 clean pass).
</commit_message>
<xml_diff>
--- a/docs/pengujian/Hasil-Pengujian-LPS-EDMS.xlsx
+++ b/docs/pengujian/Hasil-Pengujian-LPS-EDMS.xlsx
@@ -6,16 +6,18 @@
     <sheet name="Ringkasan Gabungan" sheetId="1" r:id="rId1"/>
     <sheet name="Isolasi Peran (API)" sheetId="2" r:id="rId2"/>
     <sheet name="Notulen &amp; Tindak Lanjut" sheetId="3" r:id="rId3"/>
-    <sheet name="Waktu Respons" sheetId="4" r:id="rId4"/>
-    <sheet name="Deteksi N+1" sheetId="5" r:id="rId5"/>
-    <sheet name="Beban Konkuren" sheetId="6" r:id="rId6"/>
-    <sheet name="Unggah Berkas Besar" sheetId="7" r:id="rId7"/>
-    <sheet name="Lintas Peramban" sheetId="8" r:id="rId8"/>
-    <sheet name="Integritas Basis Data" sheetId="9" r:id="rId9"/>
-    <sheet name="Arsip Dokumen (DB-D4)" sheetId="10" r:id="rId10"/>
-    <sheet name="Verifikasi Deploy Production" sheetId="11" r:id="rId11"/>
-    <sheet name="Beban Konkuren Production" sheetId="12" r:id="rId12"/>
-    <sheet name="Ringkasan Naratif" sheetId="13" r:id="rId13"/>
+    <sheet name="FR-04 Multi Peran" sheetId="4" r:id="rId4"/>
+    <sheet name="FR-08 Fase Proyek" sheetId="5" r:id="rId5"/>
+    <sheet name="Waktu Respons" sheetId="6" r:id="rId6"/>
+    <sheet name="Deteksi N+1" sheetId="7" r:id="rId7"/>
+    <sheet name="Beban Konkuren" sheetId="8" r:id="rId8"/>
+    <sheet name="Unggah Berkas Besar" sheetId="9" r:id="rId9"/>
+    <sheet name="Lintas Peramban" sheetId="10" r:id="rId10"/>
+    <sheet name="Integritas Basis Data" sheetId="11" r:id="rId11"/>
+    <sheet name="Arsip Dokumen (DB-D4)" sheetId="12" r:id="rId12"/>
+    <sheet name="Verifikasi Deploy Production" sheetId="13" r:id="rId13"/>
+    <sheet name="Beban Konkuren Production" sheetId="14" r:id="rId14"/>
+    <sheet name="Ringkasan Naratif" sheetId="15" r:id="rId15"/>
   </sheets>
 </workbook>
 </file>
@@ -409,7 +411,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G72"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1517,88 +1519,88 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>PR-01</v>
+        <v>FR-04</v>
       </c>
       <c r="B49" t="str">
-        <v>Performa</v>
+        <v>API</v>
       </c>
       <c r="C49" t="str">
-        <v>Login kelima peran di lebih dari satu peramban (mesin render berbeda)</v>
+        <v>Satu pengguna (Rina) memiliki peran berbeda di dua proyek berbeda secara bersamaan (ENGINEER di Tower A, ditambahkan sebagai TEAM_LEADER di Mall Central)</v>
       </c>
       <c r="D49" t="str">
-        <v>Berhasil login di semua peramban yang diuji</v>
+        <v>Hak akses harus berbeda per proyek dalam sesi login yang sama, bukan berlaku global untuk user itu</v>
       </c>
       <c r="E49" t="str">
-        <v>Berhasil di Chrome (Blink) dan Firefox (Gecko)</v>
+        <v>Sebelum: Rina bukan anggota Mall Central (403). Setelah ditambahkan TEAM_LEADER di Mall Central: dalam SESI LOGIN YANG SAMA, Rina bisa GET &amp; PATCH Mall Central sebagai Team Leader, TAPI PATCH ke Tower A tetap ditolak (403) karena di sana perannya masih ENGINEER</v>
       </c>
       <c r="F49" t="str">
         <v>Lolos</v>
       </c>
       <c r="G49" t="str">
-        <v>Safari (WebKit) tidak bisa diuji — programnya sendiri crash saat dibuka di laptop pengujian (kehabisan memori sistem), bukan masalah dari sisi LPS EDMS. Dua mesin render berbeda (Blink &amp; Gecko) sudah memenuhi standar minimum yang ditetapkan sebelum pengujian dimulai.</v>
+        <v>Belum pernah diuji sebelumnya — data seed hanya punya Budi selalu TEAM_LEADER dan Rina selalu ENGINEER di setiap proyek yang mereka ikuti, jadi belum ada bukti langsung resolusi peran per-proyek. Diuji dengan menambahkan peran sungguhan lewat API (Superadmin), lalu dibersihkan lagi setelah pengujian (peran tambahan dihapus).</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>PR-02</v>
+        <v>FR-08</v>
       </c>
       <c r="B50" t="str">
-        <v>Performa</v>
+        <v>API</v>
       </c>
       <c r="C50" t="str">
-        <v>Unggah dokumen di lebih dari satu peramban</v>
+        <v>Proyek baru otomatis mendapat 6 fase tetap sesuai siklus LPS (IEC 62305)</v>
       </c>
       <c r="D50" t="str">
-        <v>Berhasil di semua peramban yang diuji</v>
+        <v>Persis 6 fase, urutan tetap, semua belum aktif sampai diaktifkan manual</v>
       </c>
       <c r="E50" t="str">
-        <v>Berhasil di Chrome dan Firefox</v>
+        <v>Proyek baru dibuat lewat API sungguhan → otomatis mendapat 6 fase persis sesuai urutan (INISIASI, ASSESSMENT, DESIGN, IMPLEMENTASI, COMMISSIONING, INSPEKSI_BERKALA), semuanya isActive=false</v>
       </c>
       <c r="F50" t="str">
         <v>Lolos</v>
       </c>
       <c r="G50" t="str">
-        <v/>
+        <v>Belum pernah diuji end-to-end sebelumnya (sebelumnya hanya diverifikasi tidak langsung lewat proyek yang SUDAH difase-kan di data seed). Proyek uji dihapus lagi setelah pengujian karena masih kosong.</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>PR-03</v>
+        <v>PR-01</v>
       </c>
       <c r="B51" t="str">
         <v>Performa</v>
       </c>
       <c r="C51" t="str">
-        <v>Pencarian dokumen di lebih dari satu peramban</v>
+        <v>Login kelima peran di lebih dari satu peramban (mesin render berbeda)</v>
       </c>
       <c r="D51" t="str">
-        <v>Berhasil di semua peramban yang diuji</v>
+        <v>Berhasil login di semua peramban yang diuji</v>
       </c>
       <c r="E51" t="str">
-        <v>Berhasil di Chrome dan Firefox</v>
+        <v>Berhasil di Chrome (Blink) dan Firefox (Gecko)</v>
       </c>
       <c r="F51" t="str">
         <v>Lolos</v>
       </c>
       <c r="G51" t="str">
-        <v/>
+        <v>Safari (WebKit) tidak bisa diuji — programnya sendiri crash saat dibuka di laptop pengujian (kehabisan memori sistem), bukan masalah dari sisi LPS EDMS. Dua mesin render berbeda (Blink &amp; Gecko) sudah memenuhi standar minimum yang ditetapkan sebelum pengujian dimulai.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>PR-04</v>
+        <v>PR-02</v>
       </c>
       <c r="B52" t="str">
         <v>Performa</v>
       </c>
       <c r="C52" t="str">
-        <v>Halaman alur persetujuan dokumen tampil benar di lebih dari satu peramban</v>
+        <v>Unggah dokumen di lebih dari satu peramban</v>
       </c>
       <c r="D52" t="str">
-        <v>Tampil dengan benar di semua peramban yang diuji</v>
+        <v>Berhasil di semua peramban yang diuji</v>
       </c>
       <c r="E52" t="str">
-        <v>Tampil benar di Chrome dan Firefox</v>
+        <v>Berhasil di Chrome dan Firefox</v>
       </c>
       <c r="F52" t="str">
         <v>Lolos</v>
@@ -1609,19 +1611,19 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>PR-05</v>
+        <v>PR-03</v>
       </c>
       <c r="B53" t="str">
         <v>Performa</v>
       </c>
       <c r="C53" t="str">
-        <v>Halaman keterlacakan dokumen (panel Penelusuran Dokumen) tampil benar di lebih dari satu peramban</v>
+        <v>Pencarian dokumen di lebih dari satu peramban</v>
       </c>
       <c r="D53" t="str">
-        <v>Tampil dengan benar di semua peramban yang diuji</v>
+        <v>Berhasil di semua peramban yang diuji</v>
       </c>
       <c r="E53" t="str">
-        <v>Tampil benar di Chrome dan Firefox</v>
+        <v>Berhasil di Chrome dan Firefox</v>
       </c>
       <c r="F53" t="str">
         <v>Lolos</v>
@@ -1632,13 +1634,13 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>PR-06</v>
+        <v>PR-04</v>
       </c>
       <c r="B54" t="str">
         <v>Performa</v>
       </c>
       <c r="C54" t="str">
-        <v>Portal Client tampil benar di lebih dari satu peramban</v>
+        <v>Halaman alur persetujuan dokumen tampil benar di lebih dari satu peramban</v>
       </c>
       <c r="D54" t="str">
         <v>Tampil dengan benar di semua peramban yang diuji</v>
@@ -1655,42 +1657,42 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>PF-01</v>
+        <v>PR-05</v>
       </c>
       <c r="B55" t="str">
         <v>Performa</v>
       </c>
       <c r="C55" t="str">
-        <v>Kecepatan membuka ringkasan (dashboard) lintas proyek, dari data kecil sampai besar</v>
+        <v>Halaman keterlacakan dokumen (panel Penelusuran Dokumen) tampil benar di lebih dari satu peramban</v>
       </c>
       <c r="D55" t="str">
-        <v>Tetap cepat dan tidak memanggil query berlipat-lipat saat data bertambah</v>
+        <v>Tampil dengan benar di semua peramban yang diuji</v>
       </c>
       <c r="E55" t="str">
-        <v>Median 95-112ms di semua tingkat data (100-4.500 dokumen); jumlah pemanggilan ke basis data tetap 18 kali</v>
+        <v>Tampil benar di Chrome dan Firefox</v>
       </c>
       <c r="F55" t="str">
         <v>Lolos</v>
       </c>
       <c r="G55" t="str">
-        <v>Diukur ulang setelah perbaikan kode — tidak berubah dari sebelumnya (route ini tidak disentuh perbaikan).</v>
+        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>PF-02</v>
+        <v>PR-06</v>
       </c>
       <c r="B56" t="str">
         <v>Performa</v>
       </c>
       <c r="C56" t="str">
-        <v>Kecepatan membuka detail satu proyek beserta ringkasan kelengkapannya</v>
+        <v>Portal Client tampil benar di lebih dari satu peramban</v>
       </c>
       <c r="D56" t="str">
-        <v>Tetap cepat dan tidak memanggil query berlipat-lipat</v>
+        <v>Tampil dengan benar di semua peramban yang diuji</v>
       </c>
       <c r="E56" t="str">
-        <v>Median 56-148ms di semua tingkat data; jumlah pemanggilan ke basis data tetap 15 kali</v>
+        <v>Tampil benar di Chrome dan Firefox</v>
       </c>
       <c r="F56" t="str">
         <v>Lolos</v>
@@ -1701,65 +1703,65 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>PF-03</v>
+        <v>PF-01</v>
       </c>
       <c r="B57" t="str">
         <v>Performa</v>
       </c>
       <c r="C57" t="str">
-        <v>Kecepatan membuka daftar dokumen dalam satu proyek</v>
+        <v>Kecepatan membuka ringkasan (dashboard) lintas proyek, dari data kecil sampai besar</v>
       </c>
       <c r="D57" t="str">
-        <v>Tetap cepat dan tidak memanggil query berlipat-lipat</v>
+        <v>Tetap cepat dan tidak memanggil query berlipat-lipat saat data bertambah</v>
       </c>
       <c r="E57" t="str">
-        <v>Median 50-110ms di semua tingkat data; jumlah pemanggilan ke basis data tetap 11 kali</v>
+        <v>Median 95-112ms di semua tingkat data (100-4.500 dokumen); jumlah pemanggilan ke basis data tetap 18 kali</v>
       </c>
       <c r="F57" t="str">
         <v>Lolos</v>
       </c>
       <c r="G57" t="str">
-        <v/>
+        <v>Diukur ulang setelah perbaikan kode — tidak berubah dari sebelumnya (route ini tidak disentuh perbaikan).</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>PF-04</v>
+        <v>PF-02</v>
       </c>
       <c r="B58" t="str">
         <v>Performa</v>
       </c>
       <c r="C58" t="str">
-        <v>Kecepatan pencarian dokumen berdasarkan judul</v>
+        <v>Kecepatan membuka detail satu proyek beserta ringkasan kelengkapannya</v>
       </c>
       <c r="D58" t="str">
-        <v>Tetap cepat DAN memakai cara pencarian yang efisien, supaya tidak memburuk di masa depan</v>
+        <v>Tetap cepat dan tidak memanggil query berlipat-lipat</v>
       </c>
       <c r="E58" t="str">
-        <v>DIPERBAIKI: indeks trigram (pg_trgm) ditambahkan pada kolom judul dan kode dokumen. Dikonfirmasi lewat pemeriksaan langsung ke basis data: rencana pencarian berubah dari memindai seluruh tabel jadi memakai indeks (2,6ms, dari sebelumnya 17ms, pada 4.500 dokumen yang sama). Waktu respons lewat API juga turun (94ms → 66ms pada tingkat data yang sama)</v>
+        <v>Median 56-148ms di semua tingkat data; jumlah pemanggilan ke basis data tetap 15 kali</v>
       </c>
       <c r="F58" t="str">
         <v>Lolos</v>
       </c>
       <c r="G58" t="str">
-        <v>Migrasi basis data (CREATE EXTENSION pg_trgm + dua indeks GIN) sudah diterapkan dan diverifikasi di database uji maupun database pengembangan. Semantik pencarian tidak berubah (tetap "mengandung di mana saja", bukan "diawali dengan") — hanya cara basis data mencari yang berubah, jadi tidak ada risiko perilaku fitur berubah untuk pengguna.</v>
+        <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>PF-05</v>
+        <v>PF-03</v>
       </c>
       <c r="B59" t="str">
         <v>Performa</v>
       </c>
       <c r="C59" t="str">
-        <v>Kecepatan pencarian berdasarkan isi berkas dokumen</v>
+        <v>Kecepatan membuka daftar dokumen dalam satu proyek</v>
       </c>
       <c r="D59" t="str">
-        <v>Tetap cepat dan memakai cara pencarian yang efisien</v>
+        <v>Tetap cepat dan tidak memanggil query berlipat-lipat</v>
       </c>
       <c r="E59" t="str">
-        <v>Median naik dari 51ms ke 171ms seiring data bertambah, TAPI sudah memakai bantuan indeks pencarian khusus isi-teks yang tepat — kenaikan wajar karena hasil yang cocok makin banyak</v>
+        <v>Median 50-110ms di semua tingkat data; jumlah pemanggilan ke basis data tetap 11 kali</v>
       </c>
       <c r="F59" t="str">
         <v>Lolos</v>
@@ -1770,42 +1772,42 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>PF-06</v>
+        <v>PF-04</v>
       </c>
       <c r="B60" t="str">
         <v>Performa</v>
       </c>
       <c r="C60" t="str">
-        <v>Kecepatan membuka halaman Pusat Kepatuhan (laporan gabungan)</v>
+        <v>Kecepatan pencarian dokumen berdasarkan judul</v>
       </c>
       <c r="D60" t="str">
-        <v>Tetap cepat dan tidak memanggil query berlipat-lipat</v>
+        <v>Tetap cepat DAN memakai cara pencarian yang efisien, supaya tidak memburuk di masa depan</v>
       </c>
       <c r="E60" t="str">
-        <v>Median 91-110ms di semua tingkat data; jumlah pemanggilan ke basis data tetap 19 kali</v>
+        <v>DIPERBAIKI: indeks trigram (pg_trgm) ditambahkan pada kolom judul dan kode dokumen. Dikonfirmasi lewat pemeriksaan langsung ke basis data: rencana pencarian berubah dari memindai seluruh tabel jadi memakai indeks (2,6ms, dari sebelumnya 17ms, pada 4.500 dokumen yang sama). Waktu respons lewat API juga turun (94ms → 66ms pada tingkat data yang sama)</v>
       </c>
       <c r="F60" t="str">
         <v>Lolos</v>
       </c>
       <c r="G60" t="str">
-        <v/>
+        <v>Migrasi basis data (CREATE EXTENSION pg_trgm + dua indeks GIN) sudah diterapkan dan diverifikasi di database uji maupun database pengembangan. Semantik pencarian tidak berubah (tetap "mengandung di mana saja", bukan "diawali dengan") — hanya cara basis data mencari yang berubah, jadi tidak ada risiko perilaku fitur berubah untuk pengguna.</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>PF-07</v>
+        <v>PF-05</v>
       </c>
       <c r="B61" t="str">
         <v>Performa</v>
       </c>
       <c r="C61" t="str">
-        <v>Kecepatan membuka detail satu dokumen beserta riwayat versinya</v>
+        <v>Kecepatan pencarian berdasarkan isi berkas dokumen</v>
       </c>
       <c r="D61" t="str">
-        <v>Tetap cepat dan tidak memanggil query berlipat-lipat</v>
+        <v>Tetap cepat dan memakai cara pencarian yang efisien</v>
       </c>
       <c r="E61" t="str">
-        <v>Median 47-78ms di semua tingkat data; jumlah pemanggilan ke basis data tetap 16 kali</v>
+        <v>Median naik dari 51ms ke 171ms seiring data bertambah, TAPI sudah memakai bantuan indeks pencarian khusus isi-teks yang tepat — kenaikan wajar karena hasil yang cocok makin banyak</v>
       </c>
       <c r="F61" t="str">
         <v>Lolos</v>
@@ -1816,219 +1818,1031 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>PF-08</v>
+        <v>PF-06</v>
       </c>
       <c r="B62" t="str">
         <v>Performa</v>
       </c>
       <c r="C62" t="str">
-        <v>Ketahanan halaman ringkasan (dashboard) saat dipakai banyak orang bersamaan (5/10/20 pengguna)</v>
+        <v>Kecepatan membuka halaman Pusat Kepatuhan (laporan gabungan)</v>
       </c>
       <c r="D62" t="str">
-        <v>Tidak ada permintaan yang gagal/kehabisan waktu sampai 20 pengguna bersamaan</v>
+        <v>Tetap cepat dan tidak memanggil query berlipat-lipat</v>
       </c>
       <c r="E62" t="str">
-        <v>Diukur ulang: 0 gagal/timeout di semua tingkat beban (sebelumnya 20 dari total request gagal di 20 pengguna)</v>
+        <v>Median 91-110ms di semua tingkat data; jumlah pemanggilan ke basis data tetap 19 kali</v>
       </c>
       <c r="F62" t="str">
         <v>Lolos</v>
       </c>
       <c r="G62" t="str">
-        <v>Tidak ada perbaikan kode sesi ini yang secara langsung menyasar penyebab dugaan sebelumnya (batas sambungan basis data default) — hasil bersih kali ini kemungkinan variasi antar-percobaan, bukan bukti pasti masalahnya hilang total. Rekomendasi menaikkan batas sambungan basis data tetap disarankan untuk kepastian jangka panjang.</v>
+        <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>PF-09</v>
+        <v>PF-07</v>
       </c>
       <c r="B63" t="str">
         <v>Performa</v>
       </c>
       <c r="C63" t="str">
-        <v>Ketahanan fitur pencarian saat dipakai banyak orang bersamaan (5/10/20 pengguna)</v>
+        <v>Kecepatan membuka detail satu dokumen beserta riwayat versinya</v>
       </c>
       <c r="D63" t="str">
-        <v>Tidak ada permintaan yang gagal/kehabisan waktu sampai 20 pengguna bersamaan</v>
+        <v>Tetap cepat dan tidak memanggil query berlipat-lipat</v>
       </c>
       <c r="E63" t="str">
-        <v>Diukur ulang: 0 gagal/timeout di semua tingkat beban (sebelumnya 9 gagal di 10 pengguna, salah satunya sampai 34,8 detik)</v>
+        <v>Median 47-78ms di semua tingkat data; jumlah pemanggilan ke basis data tetap 16 kali</v>
       </c>
       <c r="F63" t="str">
         <v>Lolos</v>
       </c>
       <c r="G63" t="str">
-        <v>Catatan yang sama seperti PF-08 berlaku di sini.</v>
+        <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>PF-10</v>
+        <v>PF-08</v>
       </c>
       <c r="B64" t="str">
         <v>Performa</v>
       </c>
       <c r="C64" t="str">
-        <v>Mengunggah berkas berukuran besar (5MB, 50MB, 150MB) — sistem menjanjikan sampai 200MB</v>
+        <v>Ketahanan halaman ringkasan (dashboard) saat dipakai banyak orang bersamaan (5/10/20 pengguna)</v>
       </c>
       <c r="D64" t="str">
-        <v>Semua ukuran sampai 200MB berhasil diunggah, dengan pemakaian memori yang wajar</v>
+        <v>Tidak ada permintaan yang gagal/kehabisan waktu sampai 20 pengguna bersamaan</v>
       </c>
       <c r="E64" t="str">
-        <v>DIPERBAIKI: 50MB dan 150MB yang sebelumnya gagal total sekarang berhasil, dengan kenaikan memori mendekati nol (+0MB dan +28MB). Berkas 5MB tetap menaikkan memori cukup besar (+207MB), TAPI dibuktikan lewat pengujian pembanding bahwa ini murni biaya percobaan baca-isi-berkas (bukan bug baru, sudah ada sejak awal untuk berkas kecil)</v>
+        <v>Diukur ulang: 0 gagal/timeout di semua tingkat beban (sebelumnya 20 dari total request gagal di 20 pengguna)</v>
       </c>
       <c r="F64" t="str">
         <v>Lolos</v>
       </c>
       <c r="G64" t="str">
-        <v>Perbaikan: (1) batas ukuran body dinaikkan ke 200MB di konfigurasi, (2) proses unggah diubah jadi mengalir langsung ke disk alih-alih ditampung penuh di memori, (3) ditemukan &amp; diperbaiki juga: proses OCR latar belakang yang tadinya ikut membaca ulang berkas besar secara penuh ke memori tanpa perlu.</v>
+        <v>Tidak ada perbaikan kode sesi ini yang secara langsung menyasar penyebab dugaan sebelumnya (batas sambungan basis data default) — hasil bersih kali ini kemungkinan variasi antar-percobaan, bukan bukti pasti masalahnya hilang total. Rekomendasi menaikkan batas sambungan basis data tetap disarankan untuk kepastian jangka panjang.</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>PF-11</v>
+        <v>PF-09</v>
       </c>
       <c r="B65" t="str">
         <v>Performa</v>
       </c>
       <c r="C65" t="str">
-        <v>Apakah pencarian/tampilan data sudah dibantu "jalan pintas" pencarian (indeks) basis data yang tepat</v>
+        <v>Ketahanan fitur pencarian saat dipakai banyak orang bersamaan (5/10/20 pengguna)</v>
       </c>
       <c r="D65" t="str">
-        <v>Setiap jenis pencarian/tampilan penting memakai jalan pintas pencarian yang sesuai</v>
+        <v>Tidak ada permintaan yang gagal/kehabisan waktu sampai 20 pengguna bersamaan</v>
       </c>
       <c r="E65" t="str">
-        <v>DIPERBAIKI: sekarang 7 dari 7 pola pencarian/tampilan terbukti memakai jalan pintas yang tepat (sebelumnya 5 dari 7 — pencarian judul/kode dokumen sudah menyusul lewat indeks trigram, lihat PF-04). Dua jalan pintas tambahan yang dicurigai perlu ternyata tidak diperlukan</v>
+        <v>Diukur ulang: 0 gagal/timeout di semua tingkat beban (sebelumnya 9 gagal di 10 pengguna, salah satunya sampai 34,8 detik)</v>
       </c>
       <c r="F65" t="str">
         <v>Lolos</v>
       </c>
       <c r="G65" t="str">
-        <v/>
+        <v>Catatan yang sama seperti PF-08 berlaku di sini.</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>UX-01</v>
+        <v>PF-10</v>
       </c>
       <c r="B66" t="str">
-        <v>UI/UX</v>
+        <v>Performa</v>
       </c>
       <c r="C66" t="str">
-        <v>Halaman dokumen menampilkan versi terbaru (v2) segera setelah diunggah, tanpa perlu refresh manual</v>
+        <v>Mengunggah berkas berukuran besar (5MB, 50MB, 150MB) — sistem menjanjikan sampai 200MB</v>
       </c>
       <c r="D66" t="str">
-        <v>Versi terbaru langsung tampil</v>
+        <v>Semua ukuran sampai 200MB berhasil diunggah, dengan pemakaian memori yang wajar</v>
       </c>
       <c r="E66" t="str">
-        <v>DIPERBAIKI: sebelumnya halaman kadang masih menampilkan versi lama sampai di-refresh manual. Sekarang semua respons dari server ditandai tidak-boleh-disimpan-cache, jadi data selalu terbaru.</v>
+        <v>DIPERBAIKI: 50MB dan 150MB yang sebelumnya gagal total sekarang berhasil, dengan kenaikan memori mendekati nol (+0MB dan +28MB). Berkas 5MB tetap menaikkan memori cukup besar (+207MB), TAPI dibuktikan lewat pengujian pembanding bahwa ini murni biaya percobaan baca-isi-berkas (bukan bug baru, sudah ada sejak awal untuk berkas kecil)</v>
       </c>
       <c r="F66" t="str">
         <v>Lolos</v>
       </c>
       <c r="G66" t="str">
-        <v>Ditemukan &amp; diperbaiki di sesi ini. Sudah diverifikasi live di production.</v>
+        <v>Perbaikan: (1) batas ukuran body dinaikkan ke 200MB di konfigurasi, (2) proses unggah diubah jadi mengalir langsung ke disk alih-alih ditampung penuh di memori, (3) ditemukan &amp; diperbaiki juga: proses OCR latar belakang yang tadinya ikut membaca ulang berkas besar secara penuh ke memori tanpa perlu.</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>UX-02</v>
+        <v>PF-11</v>
       </c>
       <c r="B67" t="str">
-        <v>UI/UX</v>
+        <v>Performa</v>
       </c>
       <c r="C67" t="str">
-        <v>Tab "Riwayat" di halaman proyek menampilkan aktivitas proyek untuk Team Leader/Engineer</v>
+        <v>Apakah pencarian/tampilan data sudah dibantu "jalan pintas" pencarian (indeks) basis data yang tepat</v>
       </c>
       <c r="D67" t="str">
-        <v>Riwayat aktivitas terisi, bukan kosong</v>
+        <v>Setiap jenis pencarian/tampilan penting memakai jalan pintas pencarian yang sesuai</v>
       </c>
       <c r="E67" t="str">
-        <v>DIPERBAIKI: akar masalahnya adalah izin akses — endpoint riwayat aktivitas sebelumnya hanya mengizinkan Superadmin/Inspector, sehingga Team Leader/Engineer yang membuka riwayat PROYEK MEREKA SENDIRI selalu mendapat halaman kosong (ditolak sistem, bukan datanya memang kosong).</v>
+        <v>DIPERBAIKI: sekarang 7 dari 7 pola pencarian/tampilan terbukti memakai jalan pintas yang tepat (sebelumnya 5 dari 7 — pencarian judul/kode dokumen sudah menyusul lewat indeks trigram, lihat PF-04). Dua jalan pintas tambahan yang dicurigai perlu ternyata tidak diperlukan</v>
       </c>
       <c r="F67" t="str">
         <v>Lolos</v>
       </c>
       <c r="G67" t="str">
-        <v>Diverifikasi live di production dengan data proyek nyata — riwayat yang tadinya kosong sekarang terisi 16 catatan aktivitas.</v>
+        <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>UX-03</v>
+        <v>UX-01</v>
       </c>
       <c r="B68" t="str">
         <v>UI/UX</v>
       </c>
       <c r="C68" t="str">
-        <v>Team Leader dapat menghapus proyek miliknya sendiri (sebelumnya cuma Superadmin)</v>
+        <v>Halaman dokumen menampilkan versi terbaru (v2) segera setelah diunggah, tanpa perlu refresh manual</v>
       </c>
       <c r="D68" t="str">
-        <v>Team Leader punya opsi hapus, dengan pengaman yang sama seperti Superadmin</v>
+        <v>Versi terbaru langsung tampil</v>
       </c>
       <c r="E68" t="str">
-        <v>DITAMBAHKAN: tombol hapus proyek sekarang muncul untuk Team Leader, tetap ditolak otomatis kalau proyek sudah punya riwayat dokumen (aturan retensi yang sama, cuma diperluas SIAPA yang boleh mencoba)</v>
+        <v>DIPERBAIKI: sebelumnya halaman kadang masih menampilkan versi lama sampai di-refresh manual. Sekarang semua respons dari server ditandai tidak-boleh-disimpan-cache, jadi data selalu terbaru.</v>
       </c>
       <c r="F68" t="str">
         <v>Lolos</v>
       </c>
       <c r="G68" t="str">
-        <v>Diverifikasi: proyek kosong berhasil dihapus Team Leader, proyek berisi riwayat tetap ditolak, Engineer tetap tidak bisa sama sekali.</v>
+        <v>Ditemukan &amp; diperbaiki di sesi ini. Sudah diverifikasi live di production.</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>UX-04</v>
+        <v>UX-02</v>
       </c>
       <c r="B69" t="str">
         <v>UI/UX</v>
       </c>
       <c r="C69" t="str">
-        <v>Bagian "Kontribusi Anggota Tim" di halaman Laporan menunjukkan alasan yang jelas kalau datanya kosong</v>
+        <v>Tab "Riwayat" di halaman proyek menampilkan aktivitas proyek untuk Team Leader/Engineer</v>
       </c>
       <c r="D69" t="str">
-        <v>Ada pesan penjelasan, bukan menghilang begitu saja</v>
+        <v>Riwayat aktivitas terisi, bukan kosong</v>
       </c>
       <c r="E69" t="str">
-        <v>DIPERBAIKI: sebelumnya bagian ini langsung hilang tanpa pesan apa pun kalau tidak ada unggahan pada periode yang dipilih (default: minggu ini), terkesan seperti fitur rusak. Sekarang muncul pesan yang menyarankan memilih periode lebih panjang.</v>
+        <v>DIPERBAIKI: akar masalahnya adalah izin akses — endpoint riwayat aktivitas sebelumnya hanya mengizinkan Superadmin/Inspector, sehingga Team Leader/Engineer yang membuka riwayat PROYEK MEREKA SENDIRI selalu mendapat halaman kosong (ditolak sistem, bukan datanya memang kosong).</v>
       </c>
       <c r="F69" t="str">
         <v>Lolos</v>
       </c>
       <c r="G69" t="str">
-        <v>Perbaikan tampilan/UX, bukan perubahan logika data yang mendasarinya.</v>
+        <v>Diverifikasi live di production dengan data proyek nyata — riwayat yang tadinya kosong sekarang terisi 16 catatan aktivitas.</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>UX-05</v>
+        <v>UX-03</v>
       </c>
       <c r="B70" t="str">
         <v>UI/UX</v>
       </c>
       <c r="C70" t="str">
+        <v>Team Leader dapat menghapus proyek miliknya sendiri (sebelumnya cuma Superadmin)</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Team Leader punya opsi hapus, dengan pengaman yang sama seperti Superadmin</v>
+      </c>
+      <c r="E70" t="str">
+        <v>DITAMBAHKAN: tombol hapus proyek sekarang muncul untuk Team Leader, tetap ditolak otomatis kalau proyek sudah punya riwayat dokumen (aturan retensi yang sama, cuma diperluas SIAPA yang boleh mencoba)</v>
+      </c>
+      <c r="F70" t="str">
+        <v>Lolos</v>
+      </c>
+      <c r="G70" t="str">
+        <v>Diverifikasi: proyek kosong berhasil dihapus Team Leader, proyek berisi riwayat tetap ditolak, Engineer tetap tidak bisa sama sekali.</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>UX-04</v>
+      </c>
+      <c r="B71" t="str">
+        <v>UI/UX</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Bagian "Kontribusi Anggota Tim" di halaman Laporan menunjukkan alasan yang jelas kalau datanya kosong</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Ada pesan penjelasan, bukan menghilang begitu saja</v>
+      </c>
+      <c r="E71" t="str">
+        <v>DIPERBAIKI: sebelumnya bagian ini langsung hilang tanpa pesan apa pun kalau tidak ada unggahan pada periode yang dipilih (default: minggu ini), terkesan seperti fitur rusak. Sekarang muncul pesan yang menyarankan memilih periode lebih panjang.</v>
+      </c>
+      <c r="F71" t="str">
+        <v>Lolos</v>
+      </c>
+      <c r="G71" t="str">
+        <v>Perbaikan tampilan/UX, bukan perubahan logika data yang mendasarinya.</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>UX-05</v>
+      </c>
+      <c r="B72" t="str">
+        <v>UI/UX</v>
+      </c>
+      <c r="C72" t="str">
         <v>Pratinjau "Portal Client" oleh Team Leader benar-benar menampilkan apa yang dilihat Client, bukan tampilan Team Leader sendiri</v>
       </c>
-      <c r="D70" t="str">
+      <c r="D72" t="str">
         <v>Dokumen yang tampil di pratinjau harus sama seperti yang benar-benar dilihat Client</v>
       </c>
-      <c r="E70" t="str">
+      <c r="E72" t="str">
         <v>DIPERBAIKI: sebelumnya toggle visibilitas "Client" pada dokumen terkesan tidak berpengaruh apa-apa saat dilihat lewat Portal Client, karena halaman itu memakai hak akses Team Leader sendiri (yang bisa lihat semua), bukan mensimulasikan hak akses Client. Sekarang pratinjau benar-benar disaring sesuai yang boleh dilihat Client.</v>
       </c>
-      <c r="F70" t="str">
-        <v>Lolos</v>
-      </c>
-      <c r="G70" t="str">
+      <c r="F72" t="str">
+        <v>Lolos</v>
+      </c>
+      <c r="G72" t="str">
         <v>Diverifikasi live di production dengan data nyata: tampilan Team Leader 10 dokumen, versi pratinjau-sebagai-Client cuma 1 dokumen (sesuai yang benar-benar boleh dilihat Client).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G70"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G72"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F14"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>kode</v>
+      </c>
+      <c r="B1" t="str">
+        <v>browser</v>
+      </c>
+      <c r="C1" t="str">
+        <v>skenario</v>
+      </c>
+      <c r="D1" t="str">
+        <v>hasil</v>
+      </c>
+      <c r="E1" t="str">
+        <v>kesimpulan</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>PR-01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>chromium</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Login kelima peran</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Semua berhasil</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Lolos</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>PR-02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>chromium</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Unggah dokumen</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Berhasil</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Lolos</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>PR-03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>chromium</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Pencarian dokumen</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Berhasil</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Lolos</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>PR-04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>chromium</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Halaman persetujuan dokumen tampil</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Berhasil</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Lolos</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>PR-05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>chromium</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Panel Penelusuran Dokumen (traceability) tampil</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Berhasil</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Lolos</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>PR-06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>chromium</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Portal Client tampil</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Berhasil</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Lolos</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>PR-01</v>
+      </c>
+      <c r="B8" t="str">
+        <v>firefox</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Login kelima peran</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Semua berhasil</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Lolos</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>PR-02</v>
+      </c>
+      <c r="B9" t="str">
+        <v>firefox</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Unggah dokumen</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Berhasil</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Lolos</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>PR-03</v>
+      </c>
+      <c r="B10" t="str">
+        <v>firefox</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Pencarian dokumen</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Berhasil</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Lolos</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>PR-04</v>
+      </c>
+      <c r="B11" t="str">
+        <v>firefox</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Halaman persetujuan dokumen tampil</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Berhasil</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Lolos</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>PR-05</v>
+      </c>
+      <c r="B12" t="str">
+        <v>firefox</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Panel Penelusuran Dokumen (traceability) tampil</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Berhasil</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Lolos</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>PR-06</v>
+      </c>
+      <c r="B13" t="str">
+        <v>firefox</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Portal Client tampil</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Berhasil</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Lolos</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>PR-00</v>
+      </c>
+      <c r="B14" t="str">
+        <v>webkit</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Coba jalankan seluruh alur PR-01..06 di WebKit (Safari)</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Proses binary WebKit crash saat dibuka (\Bus error: 10\), bahkan sendirian tanpa browser lain berjalan bersamaan — dikonfirmasi memori sistem sangat menipis (&lt;10MB bebas) di mesin pengujian saat itu</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Tidak dapat diuji</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Kegagalan infrastruktur/lingkungan pengujian (bukan temuan soal aplikasinya) — bukan bug LPS EDMS. Kompatibilitas tetap diklaim cukup terbukti lewat dua mesin render berbeda (Chromium/Blink dan Firefox/Gecko), sesuai standar minimum yang ditetapkan sendiri sebelum pengujian ini dimulai.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F14"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A100"/>
+  <cols>
+    <col min="1" max="1" width="140.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v># Hasil Integritas Basis Data (Prompt 2)</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Dijalankan terhadap `lps_edms_test`, bukan produksi/dev.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>| Kode | Yang Diperiksa | Cara Pemeriksaan | Hasil | Kesimpulan | Catatan |</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>|---|---|---|---|---|---|</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>| DB-A1 | Kolom password tersimpan sebagai hash bcrypt, bukan teks biasa | Baca kolom password_hash tiap user, cocokkan pola bcrypt ($2a$/$2b$/$2y$...) | 6 user diperiksa, 0 yang BUKAN hash bcrypt | **Lolos** | Semua tersimpan sebagai hash. |</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>| DB-A2 | Tidak ada kolom lain yang menyimpan kredensial terbaca | Cari semua kolom di seluruh tabel yang namanya mengandung password/secret/token | Tidak ada kolom mencurigakan selain users.password_hash | **Lolos** |  |</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>| DB-B1 | Tepat satu versi aktif (is_current=true) per dokumen yang punya versi | GROUP BY document_id, hitung baris is_current=true, cari yang bukan tepat 1 | 0 dokumen dengan jumlah versi aktif != 1 | **Lolos** |  |</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>| DB-B2 | Nomor versi berurutan tanpa lompatan/duplikat per dokumen | Bandingkan version_number dengan ROW_NUMBER() terurut per document_id | 0 baris versi dengan nomor tidak berurutan dari total 29 baris versi | **Lolos** |  |</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>| DB-B3 | Versi lama tidak terhapus ketika versi baru dibuat | Diverifikasi lewat kode: createDocumentVersion() di document.service.ts memakai updateMany({isCurrent:false}) lalu create() versi baru — tidak ada delete() pada versi lama manapun di jalur ini | 29 baris document_versions tersimpan saat ini | **Lolos** | Diverifikasi statis (baca kode) — memicu upload versi baru lewat skrip terpisah berisiko dobel dengan Prompt 1. Bukti perilaku end-to-end sudah tercakup di skenario TL-09/EN-U2. |</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>| DB-C1 | Dokumen diarsipkan masih ada barisnya (tidak terhapus) | Hitung dokumen berstatus ARCHIVED | 0 dokumen berstatus ARCHIVED ditemukan dan bisa diambil lewat query biasa | **Lolos** | Tidak ada data uji berstatus ARCHIVED di seed standar — perlu diarsipkan satu manual untuk demonstrasi langsung (lihat TL-10). |</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>| DB-C2 | Dokumen pada proyek yang sudah diarsipkan masih terambil lewat query | Join documents ke projects, filter project.status = ARCHIVED | 2 dokumen ditemukan pada proyek berstatus ARCHIVED, semuanya terbaca normal | **Lolos** |  |</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>| DB-C3 | Tidak ada dokumen yatim (project_id menunjuk proyek yang sudah tidak ada) | Cari document.project_id yang tidak match baris manapun di projects | 0 dokumen yatim ditemukan | **Lolos** | Konsisten dengan onDelete: Cascade pada Document.project (lihat DB-D). |</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>| DB-D1 | Daftar lengkap aturan ON DELETE tiap foreign key (dari database asli, bukan asumsi skema) | Query information_schema untuk seluruh FK + referential_constraints.delete_rule | action_items.assigned_to_id→users(SET NULL) \| action_items.linked_document_id→documents(SET NULL) \| action_items.notulen_id→notulen(CASCADE) \| action_items.required_document_type_id→document_types(SET NULL) \| audit_logs.actor_id→users(SET NULL) \| audit_logs.project_id→projects(SET NULL) \| document_references.created_by_id→users(RESTRICT) \| document_references.document_id→documents(CASCADE) \| document_references.referenced_document_id→documents(CASCADE) \| document_tags.assigned_by_id→use | **Lolos** | Total 30 FK. CASCADE eksplisit: 13. Sisanya NO ACTION (setara Restrict — Prisma tidak menambah ON DELETE kalau tidak diminta eksplisit di schema.prisma). |</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>| DB-D2 | Relasi CASCADE yang berisiko menghapus dokumen/audit log tanpa sengaja | Saring FK dari DB-D1: table_name='documents' ATAU 'audit_logs' dengan delete_rule=CASCADE (baris dokumen/audit log ikut terhapus sebagai efek samping penghapusan tabel lain), lalu diverifikasi lewat perilaku nyata endpoint DELETE /api/projects/[id] (bukan cuma struktur skema) | documents.project_id→projects(CASCADE), documents.project_phase_id→project_phases(CASCADE) | **Lolos** | DIPERBAIKI (sebelumnya Gagal — lihat riwayat pengujian): documents.project_id → projects masih punya CASCADE di level skema (sengaja tidak diubah — mengubahnya jadi RESTRICT akan lebih rumit dan berisiko dibanding menjaga di level aplikasi), TAPI deleteProject() di project.service.ts sekarang memeriksa dulu sebelum menghapus: kalau ada dokumen legal_hold atau dokumen berstatus bukan DRAFT (proyek punya riwayat sungguhan), penghapusan ditolak (400) dan proyeknya tetap utuh — CASCADE di skema tidak sempat terpicu. Proyek kosong/masih draft semua tetap bisa dihapus normal. Diverifikasi ulang lewat percobaan nyata: proyek berisi dokumen APPROVED dicoba dihapus → ditolak, proyek tetap ada; proyek baru kosong dicoba dihapus → berhasil. |</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>| DB-D3 | Apakah menghapus User bisa dilakukan sama sekali, atau selalu diblokir DB kalau dia sudah beraktivitas | Daftar semua kolom FK yang menunjuk ke users, tandai mana yang NOT NULL | projects.created_by_id(wajib) \| documents.assigned_to_id(opsional) \| documents.reviewed_by_id(opsional) \| documents.uploaded_by_id(wajib) \| document_versions.created_by_id(wajib) \| audit_logs.actor_id(opsional) \| notulen.created_by_id(wajib) \| action_items.assigned_to_id(opsional) \| user_roles.user_id(wajib) \| document_versions.approved_by_id(opsional) \| document_tags.assigned_by_id(wajib) \| milestones.created_by_id(wajib) \| document_references.created_by_id(wajib) | **Lolos** | Menjelaskan kenapa sistem punya kolom is_active (nonaktifkan) alih-alih hapus baris User sungguhan — DELETE FROM users akan gagal begitu user itu sudah upload dokumen/tercatat di audit log (kolom wajib). Aman (mencegah kehilangan riwayat), tapi berarti aksi 'hapus user' di UI semestinya berarti nonaktifkan. Cocokkan dengan SA-14. |</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>| DB-E1 | Persentase kelengkapan per fase (proyek LPS Gedung Mewah Tower A) sesuai hitungan manual dari data mentah | Hitung ulang manual dari SQL mentah: dokumen wajib per fase yang APPROVED / total dokumen wajib fase. Bandingkan dengan respons NYATA GET /api/projects/[id] di server test (login sebagai Team Leader) — memvalidasi jalur permintaan penuh, bukan fungsi terisolasi. | INISIASI: manual=50%, API=50%, ASSESSMENT: manual=100%, API=100%, DESIGN: manual=0%, API=0%, IMPLEMENTASI: manual=100%, API=100%, COMMISSIONING: manual=0%, API=0%, INSPEKSI_BERKALA: manual=0%, API=0% | **Lolos** | Cocok persis. |</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>| DB-F1 | Tidak ada baris audit dengan actor kosong | COUNT(*) WHERE actor_id IS NULL | 0 dari 15 baris audit log tanpa actor | **Lolos** |  |</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>| DB-F2 | Ragam aksi yang tercatat mencakup create/edit/delete | GROUP BY action | LINK: 1, CREATE: 9, APPROVE: 2, UNLINK: 1, PHASE_CHANGE: 2 | **Lolos** | Verifikasi end-to-end (aksi lewat API lalu cek baris barunya) sudah tercakup lewat Prompt 1 dan riwayat pengujian fungsional sebelumnya — di sini hanya diverifikasi keberadaan datanya secara agregat. |</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>| DB-G1 | Tabel relasi antar-dokumen (document_references / relation_type BASED_ON, disebut Bab VI.1.5 naskah) — ada atau tidak | Cari model di schema.prisma, tabel sungguhan di database (information_schema.tables), dan endpoint API yang membacanya/menulisnya | DITEMUKAN. Tabel document_references ada di skema dan database, dengan model Prisma + enum DocumentRelationType (BASED_ON). Endpoint POST/GET/DELETE /api/documents/[id]/references sudah aktif. 0 baris referensi tersimpan saat pemeriksaan. | **Lolos** | DIPERBAIKI (sebelumnya Gagal — lihat riwayat pengujian): fitur penautan dokumen antar-fase kini benar-benar dibangun — model DocumentReference (relasi many-to-many lewat documentId/referencedDocumentId, relationType BASED_ON), endpoint API (tambah/lihat/hapus referensi per dokumen, di halaman detail dokumen), dan endpoint metrik GET /api/projects/[id]/traceability yang menghitung M-1 (Traceability Coverage) dan M-2 (Lifecycle Integration Level). Diverifikasi end-to-end: tautan berhasil dibuat, muncul di kedua arah (dokumen sumber &amp; dokumen yang dirujuk), duplikat &amp; self-reference ditolak, Client tidak bisa menautkan, metrik proyek terhitung. CATATAN PENTING: definisi M-1/M-2 di sini adalah interpretasi wajar dari nama metriknya (M-1 = %dokumen non-draft dengan minimal 1 referensi; M-2 = %pasangan fase bersebelahan yang punya dokumen saling terhubung) — BELUM dicocokkan ke rumus persis di Bab III/VI naskah skripsi, perlu diverifikasi manual oleh penulis. |</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>## Query SQL yang dipakai</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>**DB-A1**</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>```sql</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>SELECT id, password_hash FROM users</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>```</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>**DB-A2**</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>```sql</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>SELECT table_name, column_name FROM information_schema.columns WHERE column_name ILIKE '%password%' OR ILIKE '%secret%' OR ILIKE '%token%'</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>```</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>**DB-B1**</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>```sql</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>SELECT document_id, COUNT(*) FILTER (WHERE is_current) FROM document_versions GROUP BY document_id HAVING COUNT(*) FILTER (WHERE is_current) &lt;&gt; 1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>```</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>**DB-B2**</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>```sql</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>SELECT document_id, version_number, ROW_NUMBER() OVER (PARTITION BY document_id ORDER BY version_number) FROM document_versions</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>```</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>**DB-B3**</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>```sql</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>SELECT COUNT(*) FROM document_versions</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>```</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>**DB-C1**</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>```sql</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>SELECT id FROM documents WHERE status = 'ARCHIVED'</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>```</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>**DB-C2**</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>```sql</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>SELECT d.id FROM documents d JOIN projects p ON p.id=d.project_id WHERE p.status='ARCHIVED'</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>```</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>**DB-C3**</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>```sql</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>SELECT d.id FROM documents d WHERE d.project_id IS NOT NULL AND NOT EXISTS (SELECT 1 FROM projects p WHERE p.id=d.project_id)</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>```</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>**DB-D1**</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>```sql</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>SELECT tc.table_name, kcu.column_name, ccu.table_name, rc.delete_rule FROM information_schema.table_constraints ... JOIN referential_constraints</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>```</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>**DB-D2**</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>```sql</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>-- turunan DB-D1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>```</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>**DB-D3**</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>```sql</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>-- lihat cara di atas</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>```</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>**DB-E1**</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>```sql</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>-- perhitungan pembanding di SQL biasa, dicocokkan ke respons HTTP asli</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>```</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>**DB-F1**</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>```sql</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>SELECT COUNT(*) FROM audit_logs WHERE actor_id IS NULL</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>```</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>**DB-F2**</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>```sql</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>SELECT action, COUNT(*) FROM audit_logs GROUP BY action</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>```</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>**DB-G1**</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>```sql</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>SELECT table_name FROM information_schema.tables WHERE table_name ILIKE '%reference%'; SELECT COUNT(*) FROM document_references</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>```</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:A100"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F2"/>
   <sheetData>
@@ -2079,7 +2893,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F14"/>
   <sheetData>
@@ -2370,7 +3184,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L7"/>
   <sheetData>
@@ -2647,78 +3461,126 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A22"/>
+  <cols>
+    <col min="1" max="1" width="140.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Ringkasan Naratif Pengujian — LPS EDMS</v>
+        <v># Ringkasan Naratif Pengujian — LPS EDMS</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Pengujian dijalankan dalam empat lapisan: API (siapa boleh mengakses/melakukan apa), Basis Data (apakah data tersimpan dan terhubung dengan benar), Performa (kecepatan, ketahanan beban, kompatibilitas peramban), dan UI/UX (temuan dari pemakaian nyata sistem, di luar rencana pengujian awal). Seluruhnya dijalankan di lingkungan basis data terpisah — kecuali populasi data traceability dan verifikasi 5 perbaikan bug, yang memang sengaja dijalankan (dan diverifikasi) langsung di production sebagai bukti nyata untuk skripsi.</v>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Hasil akhir: 67 dari 69 titik pengujian lolos penuh.</v>
+        <v>Pengujian dijalankan dalam empat lapisan: **API** (siapa boleh mengakses/melakukan apa), **Basis Data** (apakah data tersimpan dan terhubung dengan benar), **Performa** (kecepatan, ketahanan beban, kompatibilitas peramban), dan **UI/UX** (temuan dari pemakaian nyata sistem, di luar rencana pengujian awal). Seluruhnya dijalankan di lingkungan basis data terpisah — kecuali populasi data traceability dan verifikasi 5 perbaikan bug, yang memang sengaja dijalankan (dan diverifikasi) langsung di production sebagai bukti nyata untuk skripsi.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Perkembangan sesi ini</v>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Selain 53 titik pengujian awal (yang sudah mencapai 53/53 lolos setelah serangkaian perbaikan), sesi lanjutan ini menambahkan:</v>
+        <v>**Hasil akhir: 67 dari 69 titik pengujian lolos penuh.**</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>1. FR-10 (notulen &amp; tindak lanjut) — sebelumnya belum pernah diuji sama sekali. 4 titik (FN-01, FN-02, RI-28, FN-04) menutup kekosongan ini. 3 lolos; FN-04 menemukan bug nyata: sistem tidak memeriksa sama sekali apakah tindak lanjut punya dokumen bukti sebelum diizinkan ditutup — siapa pun bisa "menyelesaikan" tindak lanjut tanpa benar-benar melampirkan bukti.</v>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2. Pengarsipan dokumen satuan (DB-D4) — sebelumnya belum pernah dibuktikan karena data uji tidak punya contoh dokumen berstatus arsip. Setelah diuji: dokumen tetap terbaca dan tidak bisa dihapus permanen lagi (sesuai ekspektasi), TAPI ternyata tidak hilang dari daftar dokumen proyek — baik di data mentah maupun tampilan web, sistem memilih tetap menampilkannya dengan label "Diarsipkan" alih-alih menyembunyikannya. Ini mungkin memang desain yang benar (transparansi), perlu dikonfirmasi ke pembimbing.</v>
+        <v>## Perkembangan sesi ini</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>3. Uji lintas peramban (NFR-07) — sebelumnya belum dijalankan. Chrome dan Firefox (dua mesin render berbeda, Blink &amp; Gecko) diuji penuh: login lima peran, unggah dokumen, pencarian, alur persetujuan, halaman keterlacakan, dan Portal Client — semua lolos di kedua peramban. Safari (WebKit) tidak bisa diuji karena programnya crash saat dibuka di laptop pengujian (kehabisan memori sistem) — ini kegagalan infrastruktur pengujian, bukan temuan tentang aplikasinya, dan dua mesin render yang berhasil diuji sudah memenuhi standar minimum yang ditetapkan sendiri sebelum pengujian dimulai.</v>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>4. Data traceability nyata sudah diisi di production. 5 tautan dokumen dibuat langsung lewat antarmuka (browser sungguhan) di proyek "LPS Rumah Sakit Harapan Bunda": Desain→Assessment Risiko, Rolling Sphere→Desain, As-Built→Desain, Log Commissioning→Checklist, dan yang paling penting — Inspeksi Berkala→Log Commissioning (kritis untuk T-02/T-12). Angka yang keluar LANGSUNG dari sistem (bukan dihitung manual): Traceability Coverage 70%, Lifecycle Integration Level 40% — keduanya di bawah target sendiri (≥80%/≥60%). Bukan karena sistemnya salah: definisi Lifecycle Integration Level di sistem ini hanya menghitung pasangan fase yang PERSIS bersebelahan, jadi tautan yang melompati satu fase (mis. As-Built di fase Commissioning berdasarkan Desain, melompati Implementasi) — meski valid dan nyata — tidak ikut terhitung. Penulis perlu memutuskan: terima apa adanya dan jelaskan keterbatasan ini di Bab VI, minta definisi metriknya diubah, atau tambah tautan lain.</v>
+        <v>Selain 53 titik pengujian awal (yang sudah mencapai 53/53 lolos setelah serangkaian perbaikan), sesi lanjutan ini menambahkan:</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>5. 5 bug nyata ditemukan dan diperbaiki dari laporan pengguna langsung (bukan dari rencana pengujian, tapi dari pemakaian sistem sesungguhnya): dokumen versi baru sempat tidak langsung tampil, tab Riwayat proyek kosong untuk Team Leader/Engineer (ternyata masalah izin akses, bukan datanya kosong), Team Leader tidak bisa menghapus proyek sendiri, bagian Kontribusi Anggota menghilang tanpa penjelasan saat kosong, dan pratinjau Portal Client oleh Team Leader tidak benar-benar mensimulasikan sudut pandang Client. Semua sudah diperbaiki dan diverifikasi langsung di production dengan data nyata.</v>
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Dua catatan yang wajib dibaca sebelum sidang</v>
+        <v>1. **FR-10 (notulen &amp; tindak lanjut) — sebelumnya belum pernah diuji sama sekali.** 4 titik (FN-01, FN-02, RI-28, FN-04) menutup kekosongan ini. 3 lolos; **FN-04 menemukan bug nyata**: sistem tidak memeriksa sama sekali apakah tindak lanjut punya dokumen bukti sebelum diizinkan ditutup — siapa pun bisa "menyelesaikan" tindak lanjut tanpa benar-benar melampirkan bukti.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Soal FN-04 (tindak lanjut bisa ditutup tanpa bukti): ini murni temuan, belum diperbaiki — perlu keputusan apakah bukti dokumen memang wajib atau memang sengaja opsional.</v>
+        <v>2. **Pengarsipan dokumen satuan (DB-D4) — sebelumnya belum pernah dibuktikan** karena data uji tidak punya contoh dokumen berstatus arsip. Setelah diuji: dokumen tetap terbaca dan tidak bisa dihapus permanen lagi (sesuai ekspektasi), TAPI ternyata **tidak hilang dari daftar dokumen proyek** — baik di data mentah maupun tampilan web, sistem memilih tetap menampilkannya dengan label "Diarsipkan" alih-alih menyembunyikannya. Ini mungkin memang desain yang benar (transparansi), perlu dikonfirmasi ke pembimbing.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Soal metrik traceability (70%/40%, di bawah target): angka ini APA ADANYA dari sistem sesuai instruksi Bab VI, bukan hasil hitung manual. Keterbatasannya sudah dijelaskan di atas dan di lampiran detail (`hasil-gabungan.csv`, kode DB-G1) — jangan sampai dikutip sebagai "sistem gagal", karena penyebabnya adalah definisi metrik yang butuh keputusan penulis, bukan bug sistem.</v>
+        <v>3. **Uji lintas peramban (NFR-07) — sebelumnya belum dijalankan.** Chrome dan Firefox (dua mesin render berbeda, Blink &amp; Gecko) diuji penuh: login lima peran, unggah dokumen, pencarian, alur persetujuan, halaman keterlacakan, dan Portal Client — semua lolos di kedua peramban. **Safari (WebKit) tidak bisa diuji** karena programnya crash saat dibuka di laptop pengujian (kehabisan memori sistem) — ini kegagalan infrastruktur pengujian, bukan temuan tentang aplikasinya, dan dua mesin render yang berhasil diuji sudah memenuhi standar minimum yang ditetapkan sendiri sebelum pengujian dimulai.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>4. **Data traceability nyata sudah diisi di production.** 5 tautan dokumen dibuat langsung lewat antarmuka (browser sungguhan) di proyek "LPS Rumah Sakit Harapan Bunda": Desain→Assessment Risiko, Rolling Sphere→Desain, As-Built→Desain, Log Commissioning→Checklist, dan yang paling penting — **Inspeksi Berkala→Log Commissioning** (kritis untuk T-02/T-12). Angka yang keluar LANGSUNG dari sistem (bukan dihitung manual): **Traceability Coverage 70%, Lifecycle Integration Level 40%** — keduanya **di bawah target sendiri** (≥80%/≥60%). Bukan karena sistemnya salah: definisi Lifecycle Integration Level di sistem ini hanya menghitung pasangan fase yang PERSIS bersebelahan, jadi tautan yang melompati satu fase (mis. As-Built di fase Commissioning berdasarkan Desain, melompati Implementasi) — meski valid dan nyata — tidak ikut terhitung. **Penulis perlu memutuskan**: terima apa adanya dan jelaskan keterbatasan ini di Bab VI, minta definisi metriknya diubah, atau tambah tautan lain.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>5. **5 bug nyata ditemukan dan diperbaiki dari laporan pengguna langsung** (bukan dari rencana pengujian, tapi dari pemakaian sistem sesungguhnya): dokumen versi baru sempat tidak langsung tampil, tab Riwayat proyek kosong untuk Team Leader/Engineer (ternyata masalah izin akses, bukan datanya kosong), Team Leader tidak bisa menghapus proyek sendiri, bagian Kontribusi Anggota menghilang tanpa penjelasan saat kosong, dan pratinjau Portal Client oleh Team Leader tidak benar-benar mensimulasikan sudut pandang Client. Semua sudah diperbaiki dan diverifikasi langsung di production dengan data nyata.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>## Dua catatan yang wajib dibaca sebelum sidang</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>**Soal FN-04 (tindak lanjut bisa ditutup tanpa bukti):** ini murni temuan, belum diperbaiki — perlu keputusan apakah bukti dokumen memang wajib atau memang sengaja opsional.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>**Soal metrik traceability (70%/40%, di bawah target):** angka ini APA ADANYA dari sistem sesuai instruksi Bab VI, bukan hasil hitung manual. Keterbatasannya sudah dijelaskan di atas dan di lampiran detail (`hasil-gabungan.csv`, kode DB-G1) — jangan sampai dikutip sebagai "sistem gagal", karena penyebabnya adalah definisi metrik yang butuh keputusan penulis, bukan bug sistem.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A22"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3659,6 +4521,84 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>kode</v>
+      </c>
+      <c r="B1" t="str">
+        <v>skenario</v>
+      </c>
+      <c r="C1" t="str">
+        <v>hasil</v>
+      </c>
+      <c r="D1" t="str">
+        <v>kesimpulan</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>FR-04</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Satu pengguna (Rina) punya peran berbeda di dua proyek berbeda secara bersamaan (ENGINEER di Tower A, TEAM_LEADER di Mall Central)</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Sebelum: Rina bukan anggota Mall Central (GET→403). Setelah ditambahkan sebagai TEAM_LEADER di Mall Central (oleh Superadmin): dalam SESI LOGIN YANG SAMA, Rina bisa GET (200) dan PATCH (200) Mall Central sebagai Team Leader, TAPI PATCH ke Tower A tetap ditolak (403) karena di sana perannya masih ENGINEER. Membuktikan resolusi peran benar-benar per-proyek, bukan flag global per-user.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Lolos</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>kode</v>
+      </c>
+      <c r="B1" t="str">
+        <v>skenario</v>
+      </c>
+      <c r="C1" t="str">
+        <v>hasil</v>
+      </c>
+      <c r="D1" t="str">
+        <v>kesimpulan</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>FR-08</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Proyek baru otomatis mendapat 6 fase tetap (INISIASI..INSPEKSI_BERKALA), semua belum aktif</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Proyek baru "Uji FR-08 1787276036318" otomatis mendapat 6 fase persis sesuai urutan siklus IEC 62305 (INISIASI → ASSESSMENT → DESIGN → IMPLEMENTASI → COMMISSIONING → INSPEKSI_BERKALA), semuanya belum aktif (isActive=false) sampai Team Leader mengaktifkannya manual.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Lolos</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J22"/>
   <sheetData>
     <row r="1">
@@ -4372,7 +5312,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G22"/>
   <sheetData>
@@ -4889,7 +5829,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L7"/>
   <sheetData>
@@ -5166,7 +6106,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H4"/>
   <sheetData>
@@ -5279,650 +6219,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F14"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>kode</v>
-      </c>
-      <c r="B1" t="str">
-        <v>browser</v>
-      </c>
-      <c r="C1" t="str">
-        <v>skenario</v>
-      </c>
-      <c r="D1" t="str">
-        <v>hasil</v>
-      </c>
-      <c r="E1" t="str">
-        <v>kesimpulan</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>PR-01</v>
-      </c>
-      <c r="B2" t="str">
-        <v>chromium</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Login kelima peran</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Semua berhasil</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Lolos</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>PR-02</v>
-      </c>
-      <c r="B3" t="str">
-        <v>chromium</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Unggah dokumen</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Berhasil</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Lolos</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>PR-03</v>
-      </c>
-      <c r="B4" t="str">
-        <v>chromium</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Pencarian dokumen</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Berhasil</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Lolos</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>PR-04</v>
-      </c>
-      <c r="B5" t="str">
-        <v>chromium</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Halaman persetujuan dokumen tampil</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Berhasil</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Lolos</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>PR-05</v>
-      </c>
-      <c r="B6" t="str">
-        <v>chromium</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Panel Penelusuran Dokumen (traceability) tampil</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Berhasil</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Lolos</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>PR-06</v>
-      </c>
-      <c r="B7" t="str">
-        <v>chromium</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Portal Client tampil</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Berhasil</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Lolos</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>PR-01</v>
-      </c>
-      <c r="B8" t="str">
-        <v>firefox</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Login kelima peran</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Semua berhasil</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Lolos</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>PR-02</v>
-      </c>
-      <c r="B9" t="str">
-        <v>firefox</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Unggah dokumen</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Berhasil</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Lolos</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>PR-03</v>
-      </c>
-      <c r="B10" t="str">
-        <v>firefox</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Pencarian dokumen</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Berhasil</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Lolos</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>PR-04</v>
-      </c>
-      <c r="B11" t="str">
-        <v>firefox</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Halaman persetujuan dokumen tampil</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Berhasil</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Lolos</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>PR-05</v>
-      </c>
-      <c r="B12" t="str">
-        <v>firefox</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Panel Penelusuran Dokumen (traceability) tampil</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Berhasil</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Lolos</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>PR-06</v>
-      </c>
-      <c r="B13" t="str">
-        <v>firefox</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Portal Client tampil</v>
-      </c>
-      <c r="D13" t="str">
-        <v>Berhasil</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Lolos</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>PR-00</v>
-      </c>
-      <c r="B14" t="str">
-        <v>webkit</v>
-      </c>
-      <c r="C14" t="str">
-        <v>Coba jalankan seluruh alur PR-01..06 di WebKit (Safari)</v>
-      </c>
-      <c r="D14" t="str">
-        <v>Proses binary WebKit crash saat dibuka (\Bus error: 10\), bahkan sendirian tanpa browser lain berjalan bersamaan — dikonfirmasi memori sistem sangat menipis (&lt;10MB bebas) di mesin pengujian saat itu</v>
-      </c>
-      <c r="E14" t="str">
-        <v>Tidak dapat diuji</v>
-      </c>
-      <c r="F14" t="str">
-        <v>Kegagalan infrastruktur/lingkungan pengujian (bukan temuan soal aplikasinya) — bukan bug LPS EDMS. Kompatibilitas tetap diklaim cukup terbukti lewat dua mesin render berbeda (Chromium/Blink dan Firefox/Gecko), sesuai standar minimum yang ditetapkan sendiri sebelum pengujian ini dimulai.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F14"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R16"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Kode</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Yang Diperiksa</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Cara Pemeriksaan</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Hasil</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Kesimpulan</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Catatan</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>DB-A1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Kolom password tersimpan sebagai hash bcrypt, bukan teks biasa</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Baca kolom password_hash tiap user, cocokkan pola bcrypt ($2a$/$2b$/$2y$...)</v>
-      </c>
-      <c r="D2" t="str">
-        <v>6 user diperiksa, 0 yang BUKAN hash bcrypt</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Lolos</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Semua tersimpan sebagai hash.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>DB-A2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Tidak ada kolom lain yang menyimpan kredensial terbaca</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Cari semua kolom di seluruh tabel yang namanya mengandung password/secret/token</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Tidak ada kolom mencurigakan selain users.password_hash</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Lolos</v>
-      </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>DB-B1</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Tepat satu versi aktif (is_current=true) per dokumen yang punya versi</v>
-      </c>
-      <c r="C4" t="str">
-        <v>GROUP BY document_id, hitung baris is_current=true, cari yang bukan tepat 1</v>
-      </c>
-      <c r="D4" t="str">
-        <v>0 dokumen dengan jumlah versi aktif != 1</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Lolos</v>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>DB-B2</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Nomor versi berurutan tanpa lompatan/duplikat per dokumen</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Bandingkan version_number dengan ROW_NUMBER() terurut per document_id</v>
-      </c>
-      <c r="D5" t="str">
-        <v>0 baris versi dengan nomor tidak berurutan dari total 29 baris versi</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Lolos</v>
-      </c>
-      <c r="F5" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>DB-B3</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Versi lama tidak terhapus ketika versi baru dibuat</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Diverifikasi lewat kode: createDocumentVersion() di document.service.ts memakai updateMany({isCurrent:false}) lalu create() versi baru — tidak ada delete() pada versi lama manapun di jalur ini</v>
-      </c>
-      <c r="D6" t="str">
-        <v>29 baris document_versions tersimpan saat ini</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Lolos</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Diverifikasi statis (baca kode) — memicu upload versi baru lewat skrip terpisah berisiko dobel dengan Prompt 1. Bukti perilaku end-to-end sudah tercakup di skenario TL-09/EN-U2.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>DB-C1</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Dokumen diarsipkan masih ada barisnya (tidak terhapus)</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Hitung dokumen berstatus ARCHIVED</v>
-      </c>
-      <c r="D7" t="str">
-        <v>0 dokumen berstatus ARCHIVED ditemukan dan bisa diambil lewat query biasa</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Lolos</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Tidak ada data uji berstatus ARCHIVED di seed standar — perlu diarsipkan satu manual untuk demonstrasi langsung (lihat TL-10).</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>DB-C2</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Dokumen pada proyek yang sudah diarsipkan masih terambil lewat query</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Join documents ke projects, filter project.status = ARCHIVED</v>
-      </c>
-      <c r="D8" t="str">
-        <v>2 dokumen ditemukan pada proyek berstatus ARCHIVED, semuanya terbaca normal</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Lolos</v>
-      </c>
-      <c r="F8" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>DB-C3</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Tidak ada dokumen yatim (project_id menunjuk proyek yang sudah tidak ada)</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Cari document.project_id yang tidak match baris manapun di projects</v>
-      </c>
-      <c r="D9" t="str">
-        <v>0 dokumen yatim ditemukan</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Lolos</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Konsisten dengan onDelete: Cascade pada Document.project (lihat DB-D).</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>DB-D1</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Daftar lengkap aturan ON DELETE tiap foreign key (dari database asli, bukan asumsi skema)</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Query information_schema untuk seluruh FK + referential_constraints.delete_rule</v>
-      </c>
-      <c r="D10" t="str">
-        <v>action_items.assigned_to_id→users(SET NULL) \</v>
-      </c>
-      <c r="E10" t="str">
-        <v>action_items.linked_document_id→documents(SET NULL) \</v>
-      </c>
-      <c r="F10" t="str">
-        <v>action_items.notulen_id→notulen(CASCADE) \</v>
-      </c>
-      <c r="G10" t="str">
-        <v>action_items.required_document_type_id→document_types(SET NULL) \</v>
-      </c>
-      <c r="H10" t="str">
-        <v>audit_logs.actor_id→users(SET NULL) \</v>
-      </c>
-      <c r="I10" t="str">
-        <v>audit_logs.project_id→projects(SET NULL) \</v>
-      </c>
-      <c r="J10" t="str">
-        <v>document_references.created_by_id→users(RESTRICT) \</v>
-      </c>
-      <c r="K10" t="str">
-        <v>document_references.document_id→documents(CASCADE) \</v>
-      </c>
-      <c r="L10" t="str">
-        <v>document_references.referenced_document_id→documents(CASCADE) \</v>
-      </c>
-      <c r="M10" t="str">
-        <v>document_tags.assigned_by_id→use</v>
-      </c>
-      <c r="N10" t="str">
-        <v>Lolos</v>
-      </c>
-      <c r="O10" t="str">
-        <v>Total 30 FK. CASCADE eksplisit: 13. Sisanya NO ACTION (setara Restrict — Prisma tidak menambah ON DELETE kalau tidak diminta eksplisit di schema.prisma).</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>DB-D2</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Relasi CASCADE yang berisiko menghapus dokumen/audit log tanpa sengaja</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Saring FK dari DB-D1: table_name='documents' ATAU 'audit_logs' dengan delete_rule=CASCADE (baris dokumen/audit log ikut terhapus sebagai efek samping penghapusan tabel lain), lalu diverifikasi lewat perilaku nyata endpoint DELETE /api/projects/[id] (bukan cuma struktur skema)</v>
-      </c>
-      <c r="D11" t="str">
-        <v>documents.project_id→projects(CASCADE), documents.project_phase_id→project_phases(CASCADE)</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Lolos</v>
-      </c>
-      <c r="F11" t="str">
-        <v>DIPERBAIKI (sebelumnya Gagal — lihat riwayat pengujian): documents.project_id → projects masih punya CASCADE di level skema (sengaja tidak diubah — mengubahnya jadi RESTRICT akan lebih rumit dan berisiko dibanding menjaga di level aplikasi), TAPI deleteProject() di project.service.ts sekarang memeriksa dulu sebelum menghapus: kalau ada dokumen legal_hold atau dokumen berstatus bukan DRAFT (proyek punya riwayat sungguhan), penghapusan ditolak (400) dan proyeknya tetap utuh — CASCADE di skema tidak sempat terpicu. Proyek kosong/masih draft semua tetap bisa dihapus normal. Diverifikasi ulang lewat percobaan nyata: proyek berisi dokumen APPROVED dicoba dihapus → ditolak, proyek tetap ada; proyek baru kosong dicoba dihapus → berhasil.</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>DB-D3</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Apakah menghapus User bisa dilakukan sama sekali, atau selalu diblokir DB kalau dia sudah beraktivitas</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Daftar semua kolom FK yang menunjuk ke users, tandai mana yang NOT NULL</v>
-      </c>
-      <c r="D12" t="str">
-        <v>projects.created_by_id(wajib) \</v>
-      </c>
-      <c r="E12" t="str">
-        <v>documents.assigned_to_id(opsional) \</v>
-      </c>
-      <c r="F12" t="str">
-        <v>documents.reviewed_by_id(opsional) \</v>
-      </c>
-      <c r="G12" t="str">
-        <v>documents.uploaded_by_id(wajib) \</v>
-      </c>
-      <c r="H12" t="str">
-        <v>document_versions.created_by_id(wajib) \</v>
-      </c>
-      <c r="I12" t="str">
-        <v>audit_logs.actor_id(opsional) \</v>
-      </c>
-      <c r="J12" t="str">
-        <v>notulen.created_by_id(wajib) \</v>
-      </c>
-      <c r="K12" t="str">
-        <v>action_items.assigned_to_id(opsional) \</v>
-      </c>
-      <c r="L12" t="str">
-        <v>user_roles.user_id(wajib) \</v>
-      </c>
-      <c r="M12" t="str">
-        <v>document_versions.approved_by_id(opsional) \</v>
-      </c>
-      <c r="N12" t="str">
-        <v>document_tags.assigned_by_id(wajib) \</v>
-      </c>
-      <c r="O12" t="str">
-        <v>milestones.created_by_id(wajib) \</v>
-      </c>
-      <c r="P12" t="str">
-        <v>document_references.created_by_id(wajib)</v>
-      </c>
-      <c r="Q12" t="str">
-        <v>Lolos</v>
-      </c>
-      <c r="R12" t="str">
-        <v>Menjelaskan kenapa sistem punya kolom is_active (nonaktifkan) alih-alih hapus baris User sungguhan — DELETE FROM users akan gagal begitu user itu sudah upload dokumen/tercatat di audit log (kolom wajib). Aman (mencegah kehilangan riwayat), tapi berarti aksi 'hapus user' di UI semestinya berarti nonaktifkan. Cocokkan dengan SA-14.</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>DB-E1</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Persentase kelengkapan per fase (proyek LPS Gedung Mewah Tower A) sesuai hitungan manual dari data mentah</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Hitung ulang manual dari SQL mentah: dokumen wajib per fase yang APPROVED / total dokumen wajib fase. Bandingkan dengan respons NYATA GET /api/projects/[id] di server test (login sebagai Team Leader) — memvalidasi jalur permintaan penuh, bukan fungsi terisolasi.</v>
-      </c>
-      <c r="D13" t="str">
-        <v>INISIASI: manual=50%, API=50%, ASSESSMENT: manual=100%, API=100%, DESIGN: manual=0%, API=0%, IMPLEMENTASI: manual=100%, API=100%, COMMISSIONING: manual=0%, API=0%, INSPEKSI_BERKALA: manual=0%, API=0%</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Lolos</v>
-      </c>
-      <c r="F13" t="str">
-        <v>Cocok persis.</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>DB-F1</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Tidak ada baris audit dengan actor kosong</v>
-      </c>
-      <c r="C14" t="str">
-        <v>COUNT(*) WHERE actor_id IS NULL</v>
-      </c>
-      <c r="D14" t="str">
-        <v>0 dari 15 baris audit log tanpa actor</v>
-      </c>
-      <c r="E14" t="str">
-        <v>Lolos</v>
-      </c>
-      <c r="F14" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>DB-F2</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Ragam aksi yang tercatat mencakup create/edit/delete</v>
-      </c>
-      <c r="C15" t="str">
-        <v>GROUP BY action</v>
-      </c>
-      <c r="D15" t="str">
-        <v>LINK: 1, CREATE: 9, APPROVE: 2, UNLINK: 1, PHASE_CHANGE: 2</v>
-      </c>
-      <c r="E15" t="str">
-        <v>Lolos</v>
-      </c>
-      <c r="F15" t="str">
-        <v>Verifikasi end-to-end (aksi lewat API lalu cek baris barunya) sudah tercakup lewat Prompt 1 dan riwayat pengujian fungsional sebelumnya — di sini hanya diverifikasi keberadaan datanya secara agregat.</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>DB-G1</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Tabel relasi antar-dokumen (document_references / relation_type BASED_ON, disebut Bab VI.1.5 naskah) — ada atau tidak</v>
-      </c>
-      <c r="C16" t="str">
-        <v>Cari model di schema.prisma, tabel sungguhan di database (information_schema.tables), dan endpoint API yang membacanya/menulisnya</v>
-      </c>
-      <c r="D16" t="str">
-        <v>DITEMUKAN. Tabel document_references ada di skema dan database, dengan model Prisma + enum DocumentRelationType (BASED_ON). Endpoint POST/GET/DELETE /api/documents/[id]/references sudah aktif. 0 baris referensi tersimpan saat pemeriksaan.</v>
-      </c>
-      <c r="E16" t="str">
-        <v>Lolos</v>
-      </c>
-      <c r="F16" t="str">
-        <v>DIPERBAIKI (sebelumnya Gagal — lihat riwayat pengujian): fitur penautan dokumen antar-fase kini benar-benar dibangun — model DocumentReference (relasi many-to-many lewat documentId/referencedDocumentId, relationType BASED_ON), endpoint API (tambah/lihat/hapus referensi per dokumen, di halaman detail dokumen), dan endpoint metrik GET /api/projects/[id]/traceability yang menghitung M-1 (Traceability Coverage) dan M-2 (Lifecycle Integration Level). Diverifikasi end-to-end: tautan berhasil dibuat, muncul di kedua arah (dokumen sumber &amp; dokumen yang dirujuk), duplikat &amp; self-reference ditolak, Client tidak bisa menautkan, metrik proyek terhitung. CATATAN PENTING: definisi M-1/M-2 di sini adalah interpretasi wajar dari nama metriknya (M-1 = %dokumen non-draft dengan minimal 1 referensi; M-2 = %pasangan fase bersebelahan yang punya dokumen saling terhubung) — BELUM dicocokkan ke rumus persis di Bab III/VI naskah skripsi, perlu diverifikasi manual oleh penulis.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R16"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>